<commit_message>
PR knowledge: cross-border PR operations LLM wiki + worklog media contacts (9) into PR team Excel
</commit_message>
<xml_diff>
--- a/PMO/业务协作_PR团队/PR团队协作表.xlsx
+++ b/PMO/业务协作_PR团队/PR团队协作表.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.核心媒体与编辑" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.周报接收人" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.专家与样机库" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.媒体联系人库" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1130,4 +1131,388 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>联系人</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>媒体</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>月流量</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>报价</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>AI合作结论</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>业务确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sarah Connor</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>bestproducts.com</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1M/月</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>免费（寄样+挂亚马逊链接）</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>建议合作：Momcozy 用户且孕期 10 周，测评/礼物指南</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Hana Amaes</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Medical News Today</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>17M/月</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>医学 blog 500欧/1500字</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>建议推进：大流量，有孕哺护肤内容经验</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Kate / Baby Chick</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>baby-chick.com</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>900万曝光/月</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>$7,500-$15,000</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>建议合作：孕期/新手妈妈受众，组合套餐</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Susey Harmer</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Today's Parent</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>600万读者/月</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>$18,500 / $11,000</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>待确认：权威强但价高，需曝光/点击数据</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Tiffany Tse</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>SheKnows</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>8000万+/月</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>待询价</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>待判断：需明确报道形式/是否挂链接/排期</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Kari Bliss</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Sophisticated Whimsy</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>未提供</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>$1,500</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>待判断：6个月新手妈妈，需补媒体资料包</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sydney Wingfield</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>The Skin (Substack)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>400-1000 views</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>$300</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>小预算尝试：skincare 场景，曝光有限</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Angela Onwuzoo</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>healthwise.punchng</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>108K/月</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>不合作：尼日利亚受众，不相关</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Hannah Payne</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>threadsbyh.com</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>无数据</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>不合作：旅游方向，不匹配</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
PMO: add PR rules confirmation sheet (ROI filter + media criteria + Earned Media logic) for business secondary confirmation
</commit_message>
<xml_diff>
--- a/PMO/业务协作_PR团队/PR团队协作表.xlsx
+++ b/PMO/业务协作_PR团队/PR团队协作表.xlsx
@@ -11,6 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.周报接收人" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.专家与样机库" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.媒体联系人库" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.规则确认" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1515,4 +1516,226 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>规则名称</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>规则内容</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AI推荐依据</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>优先级</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>业务确认</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>业务修订</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>媒体 ROI 过滤规则</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>月流量 &lt;100万 且 报价 &gt;$2,000 → 不推荐</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>工作日志筛掉 Angela Onwuzoo(108K)、Sydney Wingfield(400views) 的经验固化</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>保障曝光先问清</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>凡'保障报道/曝光'但不明确是否挂链接/赞助标注/追踪链接 → 先问清再判断</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>工作日志 Tiffany Tse(SheKnows) 待判断的经验</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>媒体判断 5 维度</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>必查：网站流量、受众地域、内容方向匹配、报价合理性、可追踪性</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>工作日志实操标准</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>海外 Earned Media 逻辑</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>海外媒体不可'买版面保出稿'，编辑决定是否报道，新闻价值&gt;品牌需求</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>一文吃透PR全貌（跨境 PR 底层逻辑）</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Pitch 个性化 + 冷却期</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>一对一 Pitch，群发模板会被编辑拉黑；同一编辑 pitch 频率过高需冷却</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>海外PR vs 国内公关（避坑）</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>PR 预算框架</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>通稿月度 3 篇、单篇 ~$2,500、月度 6-8k；外链 $1,500/月</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>工作日志预算记录，需确认是否延续</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
PR agent system prompt template (3 principles + business fill-in placeholders) + core messaging sheet for business confirmation
</commit_message>
<xml_diff>
--- a/PMO/业务协作_PR团队/PR团队协作表.xlsx
+++ b/PMO/业务协作_PR团队/PR团队协作表.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3.专家与样机库" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.媒体联系人库" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.规则确认" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6.核心信息话术" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1738,4 +1739,225 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>类别</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>内容（AI预填）</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AI推荐依据</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>业务确认</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>业务修订</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>品牌定位</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>母婴 DTC 品牌，可穿戴吸奶器 + 喂养电器</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>从竞品维度表 + 官网确认</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>核心话术-1</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Comfortable &amp; Hands-Free（舒适、免手）</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>PR 方案原文核心信息，建议确认</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>核心话术-2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>FDA Cleared / Science-backed（FDA 许可 / 科学支撑）</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>PR 方案原文核心信息，建议确认</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>核心话术-3</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>四重肽 + 9 植萃（成分浓度）</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>工作日志差异化话术，建议确认</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>核心话术-4</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>EWG 认证 + 三重专家背书</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>工作日志差异化话术，建议确认</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>禁用表述-1</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>不得承诺统一效果（'所有妈妈都适用'）</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>FTC 合规 + 母婴健康产品红线</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>禁用表述-2</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>不得使用医疗/绝对化表述（'治疗''最佳''第一'）</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>FTC 代言指南 + 医疗产品合规</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>专家背书</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>IBCLC 顾问 / 签约专家名单</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>待业务提供可对外背书专家</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>